<commit_message>
removing inner header Grade_Content
</commit_message>
<xml_diff>
--- a/TestKit/Q1/TC1/Header.xlsx
+++ b/TestKit/Q1/TC1/Header.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C709532-25FE-4719-8D12-D380E0228D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8ABC2D-CE94-4136-8EB3-F0241B469C32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -71,12 +71,6 @@
   </si>
   <si>
     <t>Type</t>
-  </si>
-  <si>
-    <t>Grade_Content</t>
-  </si>
-  <si>
-    <t>Client</t>
   </si>
 </sst>
 </file>
@@ -468,12 +462,7 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
+      <c r="A5" s="1"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>

</xml_diff>